<commit_message>
fixing the folder processing error
</commit_message>
<xml_diff>
--- a/bulk_screening_ac68c8ac.xlsx
+++ b/bulk_screening_ac68c8ac.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>80/100</t>
+          <t>85/100</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -513,12 +513,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Exceeds (Required: 3–6 years, Found: 6 years)</t>
+          <t>Exceeds (Required: 5+ years, Found: 9 years)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>['React.js', 'Javascript', 'C#', 'WebApi', '.NET', 'Linq', 'SQL Server', 'AWS', 'Agile', 'HTML', 'CSS', 'Hangfire', 'SignalR', 'Rebus', 'Entity Framework']</t>
+          <t>['React.js', 'Javascript', 'C#', 'WebApi', '.NET', 'Linq', 'SQL Server', 'AWS', 'Agile', 'HTML', 'CSS', 'Hangfire', 'SignalR', 'Rebus']</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>6 years</t>
+          <t>9 years</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Stable. Over 2 years at current company (IQVIA) and previous roles show consistent tenure.</t>
+          <t>Stable. 2 years in current company (IQVIA) with previous employment durations exceeding 2 years.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Missing hands-on experience with LLM frameworks like LangChain, LlamaIndex; experience with vector databases; and specific experience with prompt engineering.</t>
+          <t>Missing Microsoft Azure Certification.</t>
         </is>
       </c>
     </row>
@@ -580,12 +580,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Exceeds (Required: 3-6 years, Found: 13+ years)</t>
+          <t>Exceeds (Required: 5 years, Found: 13 years)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>['Typescript', 'React', 'React Native', 'Node JS', 'JavaScript', 'jQuery', 'HTML', 'CSS', 'Bootstrap', 'Redux', 'GIT', 'Material UI', 'GraphQL', 'ES6+', 'Cypress', 'BDD', 'TDD', 'AEM', 'Site core', 'Micro Frontend', 'Micro Services', 'Jest', 'PHP', 'DotNet Core', 'Web Component', 'Kubernetes', 'Docker', 'AWS Amplify']</t>
+          <t>['Typescript', 'React', 'React Native', 'JavaScript', 'jQuery', 'HTML', 'CSS', 'Bootstrap', 'Redux', 'GIT', 'Material UI', 'GraphQL', 'ES6+', 'Cypress', 'BDD', 'TDD', 'Node JS', 'Micro Frontend', 'Micro Services', 'Jest', 'PHP', 'DotNet Core', 'Web Component', 'Kubernetes', 'Docker', 'AWS Amplify', 'ASP.net', 'Postgres', 'MongoDB', 'Redis']</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>13+ years</t>
+          <t>13 years</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Stable. Current role for 1 year 6 months, previous role for 2 years 9 months.</t>
+          <t>Stable. Current role for 1 year 6 months at Espire Infolabs Pvt. Ltd.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Missing specific experience with LLM frameworks like LangChain, LlamaIndex, or similar; no mention of Generative AI applications.</t>
+          <t>Missing specific mention of Microsoft Azure Certification</t>
         </is>
       </c>
     </row>
@@ -637,22 +637,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>50/100</t>
+          <t>30/100</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Completed certification of ISO 27001:2022 Information security management system, Cybersecurity &amp; Digital Forensics from IIT KOTA, Oracle cloud infrastructure foundation 2021 Associate, Training on McAfee DLP Policy monitoring from Shivalik Bank, Webinar on Cyber warfare, cyber security and cyber citizenship by BVICAM</t>
+          <t>Completed certification of ISO 27001:2022 Information security management system</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Exceeds (Required: 3-6+ years, Found: 8+ years)</t>
+          <t>Exceeds (Required: 5 years, Found: 8 years)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>['Information Security', 'DLP Monitoring', 'Policy Creation', 'IT Risk Assessment', 'Data Security', 'IT Act', 'IT Governance', 'Internal IT Audit', 'Cybersecurity Training', 'Incident Analysis', 'Cyber Security Management', 'Active Directory Management', 'Data Privacy', 'Vulnerability Assessment', 'Trend Micro Management', 'McAfee Management', 'Microsoft Cloud Management', 'ITIL Practices']</t>
+          <t>['DLP monitoring', 'Implementation', 'Policy creation', 'IT Risk assessment', 'Data security', 'Cybersecurity training', 'Trend Micro Antivirus', 'Active Directory Management', 'Group policy management', 'Information security risk management', 'Patch management', 'Microsoft purview Email DLP management']</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>08+ Years</t>
+          <t>8 years</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Stable. Tenure at current company (ORIX Corporation India Limited) yet to be assessed as role started Sep 2025.</t>
+          <t>Stable. Currently employed at ORIX Corporation with ongoing tenure.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Missing direct experience with LLM frameworks like LangChain, deployment of AI solutions on cloud platforms, and integration of LLM APIs.</t>
+          <t>Missing specific experience in Python development, Microsoft Azure Certification, frontend technologies like React/Angular/Vue.js.</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>70/100</t>
+          <t>85/100</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Exceeds (Required: 3–6+ years, Found: Over 7 Years)</t>
+          <t>Exceeds (Required: 5 years, Found: Over 7 Years)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>['MS SQL', 'Mongo DB', 'HTML5', 'CSS', 'REST', '.Net Core', 'C#', 'JavaScript', 'Messaging Queue', 'Git', 'GCP', 'Azure Devops', 'Node JS', 'React JS', 'Docker', 'Microservices']</t>
+          <t>['Full Stack', 'Development', 'Technology Lead', 'Application Analyst', 'Banking', 'Healthcare', 'Ecommerce', 'MS SQL', 'Mongo DB', 'HTML5', 'CSS', 'REST', '.Net Core', 'C#', 'JavaScript', 'Messaging Queue', 'Git', 'GCP', 'Azure Devops', 'Node JS', 'React JS', 'Docker', 'Microservices']</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Not enough information available for stability assessment</t>
+          <t>Not enough information to assess stability. No clear company tenures provided.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Missing specific experience with Generative AI, LLM frameworks, prompt engineering, and integration of LLM APIs.</t>
+          <t>Missing specific experience with Python frameworks such as Django or Flask, and Azure certification.</t>
         </is>
       </c>
     </row>
@@ -771,22 +771,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>85/100</t>
+          <t>80/100</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Project Management Professional- PMP, Certified Ethical Hacker- CEH, Certified Information Security Manager -CISM, Lead Auditor ISO 27001: ISMS, ITIL Intermediate - OSA &amp; V3 Foundation Certified, IBM- Certified Organization and Professional ethics, IBM Certified Delivery Manager, Microsoft Certified Professional -MCP</t>
+          <t>Microsoft Certified Professional - MCP</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Exceeds (Required: 3-6+ years, Found: 16 years)</t>
+          <t>Exceeds (Required: 5+ years, Found: 16 years)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>['Cybersecurity', 'IAM', 'Infrastructure Security', 'Governance', 'Risk Management', 'Project Management', 'Service Delivery', 'Incident Management', 'Data Protection', 'Compliance Audits', 'Stakeholder Communication', 'Access Control', 'Zero Trust', 'SSO', 'MFA', 'RBAC', 'Audits', 'Change Management', 'Performance Improvement']</t>
+          <t>['IT Leadership &amp; Program Management', 'IT Project &amp; Service Delivery', 'ITSM (Jira)', 'Change Management', 'Incident Management', 'Problem Management', 'KPI &amp; SLA Governance', 'Governance, Risk &amp; Compliance', 'IT Audits &amp; Regulatory Compliance', 'Cybersecurity &amp; IAM Operations', 'Identity &amp; Access Control', 'Security Standards Alignment', 'Strategy &amp; Business Management', 'Vendor &amp; Contract Management', 'Performance Improvement Plans', 'Agile &amp; Scrum', 'Stakeholder Communication', 'Employee Engagement &amp; Adaptability']</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Stable. Tenure at HSBC not less than 2 years.</t>
+          <t>Stable. Multiple roles at large organizations, tenure not specified.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Missing specific experience with LLM frameworks, APIs integration into backend systems, and experience working with vector databases.</t>
+          <t>Missing specific experience in Python frameworks (Django, Flask, FastAPI) and frontend technologies (React, Angular, Vue.js).</t>
         </is>
       </c>
     </row>
@@ -838,7 +838,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>80/100</t>
+          <t>85/100</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -848,12 +848,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Exceeds (Required: 3-6 years, Found: 6.5 years)</t>
+          <t>Exceeds (Required: 5 years, Found: 6.5 years)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>['Oracle Applications R12', 'Financial module', 'Procure-to-pay', 'Core HRMS', 'PL/SQL', 'SQL', 'API Testing with Postman', 'Oracle Apex', 'E-Business Suite', 'RICE Components', 'Oracle Forms', 'Advanced SQL concepts', 'XML Reports', 'Oracle Financial Module (GL)', 'Troubleshooting', 'Form personalization', 'Developing Concurrent Programs']</t>
+          <t>['Python', 'SQL', 'PL/SQL', 'Oracle Applications R12', 'Oracle Apex', 'REST APIs', 'Postman', 'HTML', 'CSS', 'JavaScript', 'Oracle Core HRMS', 'Oracle Financial Module', 'Git', 'Agile', 'Unix', 'Java', 'PHP', 'DBMS', 'RDBMS']</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Stable. 6.5 years across various projects; tenure is acceptable.</t>
+          <t>Stable. 6.5 years of total experience across multiple roles.</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Missing experience with Generative AI, LLM frameworks, and specific knowledge of tools like Docker, Kubernetes, and vector databases.</t>
+          <t>Missing explicit Microsoft Azure Certification, experience in modern architectures and cloud-based solutions.</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>70/100</t>
+          <t>60/100</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -915,12 +915,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Exceeds (Required: 3–6+, Found: 15 years)</t>
+          <t>Exceeds (Required: 5 years, Found: 15+ years)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>['Cybersecurity Project Management', 'Firewall Migration', 'Vulnerability Assessment &amp; Remediation', 'IT Infrastructure Delivery', 'Stakeholder &amp; Vendor Management', 'Cloud &amp; Data Center Management', 'Network Security &amp; Governance', 'Risk Mitigation &amp; Compliance', 'Agile &amp; Waterfall Methodologies', 'Zero Trust Architecture', 'IAM / PAM / SSO', 'GRC (Governance, Risk &amp; Compliance)', 'ServiceNow', 'Jira', 'MS Visio']</t>
+          <t>['Cybersecurity Project Management', 'Firewall Migration (Checkpoint to Fortinet)', 'Vulnerability Assessment &amp; Remediation', 'IT Infrastructure Delivery', 'Stakeholder &amp; Vendor Management', 'Cloud &amp; Data Center Management', 'Network Security &amp; Governance', 'Risk Mitigation &amp; Compliance (NIST, ISO 27001)', 'Agile &amp; Waterfall Methodologies', 'Zero Trust Architecture', 'IAM / PAM / SSO', 'GRC (Governance, Risk &amp; Compliance)', 'ServiceNow', 'Jira', 'MS Visio']</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>15 years</t>
+          <t>15+ years</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -950,17 +950,17 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Identified a brief gap (Aug–Sep 2014) due to transition from Virtela to Rolta.</t>
+          <t>Brief gap (Aug–Sep 2014) due to transition from Virtela to Rolta.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Stable. 15 years across various companies with notable tenures.</t>
+          <t>Stable. Most recent role at BCT Consulting lasted from Feb 2021 to Nov 2023.</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Missing hands-on experience with LLM frameworks, specific experience in integrating GenAI capabilities, and familiarity with vector databases.</t>
+          <t>Missing Azure certification. No mention of Python or full-stack development experience.</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>85/100</t>
+          <t>80/100</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -982,12 +982,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Exceeds (Required: 3-6+ years, Found: 7 years)</t>
+          <t>Exceeds (Required: 5 years, Found: 7 years)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>['Gen AI', 'Cloud', 'Cybersecurity', 'Supply Chain Management (SCM)', 'Agile/Scrum Methodology', 'Sprint Planning', 'Requirements Gathering', 'User Story Writing', 'GAP Analysis', 'Stakeholder Management', 'UAT/SIT Test Planning', 'Defect Tracking', 'Jira', 'Confluence', 'ADO', 'Salesforce', 'SailPoint', 'Label Studio', 'AI Data Foundry', 'Azure']</t>
+          <t>['Agile', 'Scrum', 'Project Management', 'Confluence', 'Jira', 'ADO', 'Salesforce', 'SailPoint', 'Label Studio', 'AI Data Foundry', 'Azure', 'Cybersecurity', 'IAM', 'Gen AI', 'Cloud Migration', 'Supply Chain Management', 'Requirements Gathering', 'User Story Writing', 'GAP Analysis', 'Stakeholder Management', 'UAT/SIT Test Planning', 'Defect Tracking']</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Stable. Several roles with long tenures.</t>
+          <t>Stable. Most recent tenure at Centific was 3 years.</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Missing specific hands-on experience with LLM frameworks like LangChain, LlamaIndex or experience with vector databases.</t>
+          <t>Missing specific hands-on experience with Python frameworks like Django, Flask, or FastAPI and no mention of Microsoft Azure Certification.</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>20/100</t>
+          <t>40/100</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1049,12 +1049,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Exceeds (Required: 3-6+ years, Found: 8+ years)</t>
+          <t>Exceeds (Required: 5 years, Found: 8+ years)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>['Agile', 'Manual Testing', 'Test Documentation', 'Database testing', 'Functional Testing', 'System Testing', 'Regression Testing', 'Sanity Testing', 'Smoke Testing', 'Integration Testing', 'JIRA', 'Phabricator', 'ALM', 'Oracle SQL Developer']</t>
+          <t>['Manual Testing', 'Agile', 'Web-based and Mobile applications testing', 'Test Documentation', 'Bug reporting', 'Database testing', 'Functional Testing', 'System Testing', 'Regression Testing', 'Sanity Testing', 'Smoke Testing', 'Integration Testing', 'Test Management tools (JIRA, Phabricator, ALM)', 'SQL']</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Stable. Current role at Tata Consultancy Services since Jan 2022.</t>
+          <t>Stable. 1.5 years at current company (Tata Consultancy Services). Previous role was 4.5 years at Accenture.</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Missing experience in LLM frameworks, integrating GenAI capabilities, backend services development, and specific knowledge of vector databases.</t>
+          <t>Missing experience in Python development, full-stack development, Azure certification, and specific frameworks like Django or Flask.</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>65/100</t>
+          <t>80/100</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1116,12 +1116,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Exceeds (Required: 3-6+ years, Found: 10 years 0 months)</t>
+          <t>Exceeds (Required: 5 years, Found: 10 years)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>['Streamlined QA workflows', 'Cross-functional collaboration', 'Quality metrics monitoring', 'AI/ML testing', 'API automation', 'Python', 'SQL', 'REST APIs', 'UAT execution', 'Mobile application testing', 'Performance testing', 'CI/CD integration', 'Defect triage', 'Test planning', 'Automation efficiency', 'Postman', 'JIRA', 'Agile methodology']</t>
+          <t>['Python', 'Postman', 'SQL', 'REST APIs', 'OCR', 'AI/ML', 'Salesforce CRM', 'AEM', 'Android Studio', 'Xcode', 'Charles Proxy', 'Jenkins', 'SOAP UI', 'Perfecto', 'QTest', 'GIT', 'Mobile QA', 'API Testing', 'Test Leadership', 'Agile Alignment', 'Automation Efficiency']</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>10 years 0 months</t>
+          <t>10 years</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Stable. No role less than 2 years.</t>
+          <t>Stable. 10 years with multiple employers, no role under 2 years.</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Missing direct experience with GenAI/LLM-based applications and specific tools/technologies in the JD like LangChain, FAISS, Pinecone, prompt engineering, and various cloud platforms.</t>
+          <t>Missing Microsoft Azure Certification and direct front-end technologies experience (React/Angular/Vue).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed the errors in folder processing
</commit_message>
<xml_diff>
--- a/bulk_screening_ac68c8ac.xlsx
+++ b/bulk_screening_ac68c8ac.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>80/100</t>
+          <t>85/100</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>['AWS S3', 'AWS Lambda', 'Web API', 'C#', 'React.js', '.NET', 'SQL Server', 'Hangfire', 'SignalR', 'Rebus', 'Agile', 'LINQ', 'HTML', 'CSS', 'Javascript']</t>
+          <t>['React.js', 'Javascript', 'C#', 'WebApi', '.NET', 'Linq', 'SQL Server', 'AWS', 'Agile', 'HTML', 'CSS', 'Hangfire', 'SignalR', 'Rebus', 'ML']</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Stable. 8 years total across 4 companies.</t>
+          <t>Stable. 4 employers over 8 years, with increasing responsibilities.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Missing specific experience with real-time analytics, advanced AI/ML enablement, cybersecurity frameworks like NIST CSF or MITRE ATT&amp;CK.</t>
+          <t>Missing specific experience with cybersecurity data sources and compliance standards.</t>
         </is>
       </c>
     </row>
@@ -580,12 +580,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Exceeds (Required: 8 years, Found: 13+ years)</t>
+          <t>Exceeds (Required: 8 years, Found: 13 years)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>['Typescript', 'React', 'React Native', 'JavaScript', 'jQuery', 'HTML', 'CSS', 'Bootstrap', 'Redux', 'GIT', 'Material UI', 'GraphQL', 'ES6+', 'Cypress', 'BDD', 'TDD', 'AEM', 'Sitecore', 'Node JS', 'Micro Frontend', 'Micro Services', 'Jest', 'PHP', 'DotNet Core', 'Web Component', 'Kubernetes', 'Docker', 'AWS Amplify', 'ASP.net', 'Postgres', 'MongoDB', 'Redis']</t>
+          <t>['React JS', 'React Native', 'JavaScript', 'jQuery', 'HTML', 'CSS', 'Bootstrap', 'Redux', 'GIT', 'Material UI', 'GraphQL', 'Cypress', 'BDD', 'TDD', 'AEM', 'Site core', 'Node JS', 'Micro Frontend', 'Micro Services', 'Jest', 'PHP', 'DotNet Core', 'Web Component', 'Kubernetes', 'Docker', 'AWS Amplify', 'ASP.net', 'Postgres', 'MongoDB', 'Redis']</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>13+ years</t>
+          <t>13 years</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -615,17 +615,17 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Identified a gap of 4 months between pandemic freelancing and prior experience, and 1 year 8 months from the last official role to current.</t>
+          <t>Identified a gap between graduation (2008) and first listed job (May 2016).</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Instability noted with multiple employers in less than 2 years tenure. Only 3 employers with tenures over 1 year.</t>
+          <t>Stable. 1.5 years at current company (Espire Infolabs Pvt. Ltd) and previous role at ACET Infotech for 2.9 years.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Missing specific experience in cybersecurity data sources, secure data pipelines in AWS, deep understanding of cloud security principles, and lack of leadership roles in cybersecurity context.</t>
+          <t>Missing specific experience in AWS services like Lambda, Glue, Redshift, Athena, IAM; cybersecurity-specific experience; compliance with relevant standards (NIST, ISO 27001).</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Completed certification of ISO 27001:2022 Information security management system, Cybersecurity &amp; Digital Forensics from IIT KOTA, Oracle cloud infrastructure foundation 2021 Associate, Training on McAfee DLP Policy monitoring from Shivalik Bank, Webinar on Cyber warfare, cyber security and cyber citizenship by BVICAM</t>
+          <t>Completed certification of ISO 27001:2022 Information security management system; Cybersecurity &amp; Digital Forensics from IIT KOTA; Oracle cloud infrastructure foundation 2021 Associate; Training on McAfee DLP Policy monitoring from Shivalik Bank; Webinar on Cyber warfare, cyber security and cyber citizenship by BVICAM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>['Information Security', 'DLP Monitoring', 'Policy Creation', 'IT Risk Assessment', 'Data Security', 'Cyber Security Training', 'Incident Analysis', 'Vulnerability Assessment', 'Active Directory Management', 'Group Policy Management', 'Compliance Reporting', 'Endpoint Management', 'Trend Micro Antivirus', 'McAfee DLP', 'Cybersecurity Audits', 'Regulatory Requirements']</t>
+          <t>['information security', 'DLP monitoring', 'implementation', 'policy creation', 'risk assessment', 'data security', 'internal IT Audit', 'ISO 27001:2022', 'audit compliance', 'Cybersecurity training', 'Sentinelone EDR', 'Trellix EPO', 'Trend Micro Antivirus', 'Mobile Security Management', 'AD and group policy management', 'DPDP ACT 2023', 'Microsoft Purview Email DLP management', 'McAfee DLP', 'CASB', 'patch management', 'incident analysis', 'cybersecurity tools', 'security audit', 'vulnerability assessment', 'IT security &amp; Audit policy (CSITE)', 'incident management', 'technical support', 'vendor management', 'Oracle cloud infrastructure']</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Stable. 4 years at current company (ORIX Corporation India Limited) and 4 years in previous employment.</t>
+          <t>Stable. Over 2 years at ORIX Corporation India Limited.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Missing hands-on experience with AWS services such as Lambda, Glue, Redshift, Athena, S3, IAM, KMS.</t>
+          <t>Missing specific experience in AWS services such as Lambda, Glue, Redshift, Athena, IAM, KMS, and knowledge of cybersecurity frameworks like NIST CSF, MITRE ATT&amp;CK.</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>60/100</t>
+          <t>50/100</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Not enough information to determine stability due to lack of employment history</t>
+          <t>Not enough information for stability assessment</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Missing specific experience in AWS, cyber security data sources, and relevant certifications.</t>
+          <t>Missing experience with AWS services, cybersecurity knowledge, and compliance standards.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed the errors in by adding logs and files for ogging the errors and some changes in the ngnix file also
</commit_message>
<xml_diff>
--- a/bulk_screening_ac68c8ac.xlsx
+++ b/bulk_screening_ac68c8ac.xlsx
@@ -513,12 +513,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Meets (Required: 8 years, Found: 8 years)</t>
+          <t>Meets (Required: 8+ years, Found: 8 years)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>['React.js', 'Javascript', 'C#', 'WebApi', '.NET', 'Linq', 'SQL Server', 'AWS', 'Agile', 'HTML', 'CSS', 'Hangfire', 'SignalR', 'Rebus', 'ML']</t>
+          <t>['React.js', 'Javascript', 'C#', 'WebApi', '.NET', 'Linq', 'SQL Server', 'AWS', 'Agile', 'HTML', 'CSS', 'Hangfire', 'SignalR', 'ML', 'Rebus', 'Entity Framework']</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Stable. 4 employers over 8 years, with increasing responsibilities.</t>
+          <t>Stable. 3 roles in last 8 years with latest role held since Mar 2025.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Missing specific experience with cybersecurity data sources and compliance standards.</t>
+          <t>Missing explicit experience in cybersecurity frameworks and direct mention of tools such as Lambda, Glue, Redshift, Athena, IAM, KMS.</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>70/100</t>
+          <t>60/100</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -580,12 +580,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Exceeds (Required: 8 years, Found: 13 years)</t>
+          <t>Exceeds (Required: 8+ years, Found: 13 years)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>['React JS', 'React Native', 'JavaScript', 'jQuery', 'HTML', 'CSS', 'Bootstrap', 'Redux', 'GIT', 'Material UI', 'GraphQL', 'Cypress', 'BDD', 'TDD', 'AEM', 'Site core', 'Node JS', 'Micro Frontend', 'Micro Services', 'Jest', 'PHP', 'DotNet Core', 'Web Component', 'Kubernetes', 'Docker', 'AWS Amplify', 'ASP.net', 'Postgres', 'MongoDB', 'Redis']</t>
+          <t>['Typescript', 'React', 'React Native', 'JavaScript', 'jQuery', 'HTML', 'CSS', 'Bootstrap', 'Redux', 'GIT', 'Material UI', 'GraphQL', 'ES6+', 'Cypress', 'BDD', 'TDD', 'AEM', 'Site core', 'Node JS', 'Micro Frontend', 'Micro Services', 'Jest', 'PHP', 'DotNet Core', 'Web Component', 'Kubernetes', 'Docker', 'AWS Amplify', 'ASP.net', 'Postgres', 'MongoDB', 'Redis', 'Word Press', 'PHP', 'Drupal', 'Maganto']</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -615,17 +615,17 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Identified a gap between graduation (2008) and first listed job (May 2016).</t>
+          <t>Identified a gap between Dec 2019 and March 2020 due to freelancing experience.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Stable. 1.5 years at current company (Espire Infolabs Pvt. Ltd) and previous role at ACET Infotech for 2.9 years.</t>
+          <t>Stable. No role is consistently &lt;2 years.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Missing specific experience in AWS services like Lambda, Glue, Redshift, Athena, IAM; cybersecurity-specific experience; compliance with relevant standards (NIST, ISO 27001).</t>
+          <t>Lacks specific experience with AWS services such as Lambda, Glue, Redshift, Athena, IAM, KMS and Cybersecurity frameworks.</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>['information security', 'DLP monitoring', 'implementation', 'policy creation', 'risk assessment', 'data security', 'internal IT Audit', 'ISO 27001:2022', 'audit compliance', 'Cybersecurity training', 'Sentinelone EDR', 'Trellix EPO', 'Trend Micro Antivirus', 'Mobile Security Management', 'AD and group policy management', 'DPDP ACT 2023', 'Microsoft Purview Email DLP management', 'McAfee DLP', 'CASB', 'patch management', 'incident analysis', 'cybersecurity tools', 'security audit', 'vulnerability assessment', 'IT security &amp; Audit policy (CSITE)', 'incident management', 'technical support', 'vendor management', 'Oracle cloud infrastructure']</t>
+          <t>['Information Security', 'DLP Monitoring', 'Policy Creation', 'IT Risk Assessment', 'Data Security', 'IT Governance', 'Internal IT Audit', 'Cybersecurity Audit', 'Incident Management', 'Active Directory Management', 'Vulnerability Assessment', 'Patch Management', 'Trend Micro Antivirus', 'McAfee DLP', 'Implementation of Cyber Security Training', 'Data Privacy Management']</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>8340516142/9122420165</t>
+          <t>8340516142</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>ORIX Corporation India Limited (HO-New Delhi)</t>
+          <t>ORIX Corporation India Limited</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Stable. Over 2 years at ORIX Corporation India Limited.</t>
+          <t>Stable. Continuous employment with last two roles totaling more than 5 years.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Missing specific experience in AWS services such as Lambda, Glue, Redshift, Athena, IAM, KMS, and knowledge of cybersecurity frameworks like NIST CSF, MITRE ATT&amp;CK.</t>
+          <t>Missing experience with AWS services such as Lambda, Glue, Redshift, Athena, S3, IAM, KMS and experience in AI/ML applications.</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>50/100</t>
+          <t>60/100</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Not enough information for stability assessment</t>
+          <t>Not enough information to assess stability</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Missing experience with AWS services, cybersecurity knowledge, and compliance standards.</t>
+          <t>Missing experience with AWS, cybersecurity frameworks, and specific data engineering tools like AWS Lambda, Glue, Redshift, Athena, KMS.</t>
         </is>
       </c>
     </row>

</xml_diff>